<commit_message>
2days in one day
</commit_message>
<xml_diff>
--- a/12620127.xlsx
+++ b/12620127.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Daily Routine LPU\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CE4A7B5-4D92-40B9-9CE7-37EEB3C356C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2398B49-6161-4FF2-BDE3-9E06566C09E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="70">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -243,7 +243,7 @@
     <t xml:space="preserve">The day was a west </t>
   </si>
   <si>
-    <t>2026-0825</t>
+    <t>not feel like to study</t>
   </si>
 </sst>
 </file>
@@ -1358,10 +1358,10 @@
         <v>0</v>
       </c>
       <c r="D13" s="14">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="E13" s="14">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F13" s="14">
         <v>0</v>
@@ -1374,11 +1374,11 @@
       </c>
       <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v>930</v>
+        <v>670</v>
       </c>
       <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v>510</v>
+        <v>770</v>
       </c>
       <c r="K13" s="16" t="s">
         <v>49</v>
@@ -1404,10 +1404,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="14">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="E14" s="14">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F14" s="14">
         <v>240</v>
@@ -1420,11 +1420,11 @@
       </c>
       <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v>980</v>
+        <v>830</v>
       </c>
       <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v>460</v>
+        <v>610</v>
       </c>
       <c r="K14" s="16" t="s">
         <v>49</v>
@@ -1440,89 +1440,157 @@
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="13">
+        <v>46259</v>
+      </c>
+      <c r="B15" s="14">
+        <v>400</v>
+      </c>
+      <c r="C15" s="14">
+        <v>0</v>
+      </c>
+      <c r="D15" s="14">
+        <v>0</v>
+      </c>
+      <c r="E15" s="14">
+        <v>0</v>
+      </c>
+      <c r="F15" s="14">
+        <v>300</v>
+      </c>
+      <c r="G15" s="14">
+        <v>5</v>
+      </c>
+      <c r="H15" s="14">
+        <v>300</v>
+      </c>
+      <c r="I15" s="15">
+        <f t="shared" si="0"/>
+        <v>1000</v>
+      </c>
+      <c r="J15" s="15">
+        <f t="shared" si="1"/>
+        <v>440</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N15" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="str">
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A16" s="13">
+        <v>46260</v>
+      </c>
+      <c r="B16" s="14">
+        <v>380</v>
+      </c>
+      <c r="C16" s="14">
+        <v>0</v>
+      </c>
+      <c r="D16" s="14">
+        <v>0</v>
+      </c>
+      <c r="E16" s="14">
+        <v>0</v>
+      </c>
+      <c r="F16" s="14">
+        <v>300</v>
+      </c>
+      <c r="G16" s="14">
+        <v>5</v>
+      </c>
+      <c r="H16" s="14">
+        <v>300</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="15" t="str">
+        <v>980</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
-      <c r="N15" s="17"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="17"/>
+        <v>460</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N16" s="17" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="13"/>
+      <c r="A17" s="13">
+        <v>46261</v>
+      </c>
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15" t="str">
+      <c r="F17" s="14">
+        <v>360</v>
+      </c>
+      <c r="G17" s="14">
+        <v>6</v>
+      </c>
+      <c r="H17" s="14">
+        <v>300</v>
+      </c>
+      <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="15" t="str">
+        <v>660</v>
+      </c>
+      <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
-      <c r="N17" s="17"/>
+        <v>780</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
+      <c r="A18" s="13">
+        <v>46262</v>
+      </c>
       <c r="B18" s="14"/>
       <c r="C18" s="14"/>
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
+      <c r="F18" s="14">
+        <v>420</v>
+      </c>
+      <c r="G18" s="14">
+        <v>7</v>
+      </c>
       <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>420</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
+        <v>1020</v>
       </c>
       <c r="K18" s="16"/>
       <c r="L18" s="16"/>

</xml_diff>